<commit_message>
SEGUNDA PARTE Banco Tabajara
</commit_message>
<xml_diff>
--- a/base_BANCO_TABAJARA.xlsx
+++ b/base_BANCO_TABAJARA.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,16 +478,14 @@
       <c r="E2" t="n">
         <v>400</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>'00</t>
-        </is>
+      <c r="F2" t="n">
+        <v>57.5</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -510,10 +508,8 @@
       <c r="E3" t="n">
         <v>401</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>'01</t>
-        </is>
+      <c r="F3" t="n">
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -525,7 +521,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Douglas</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -534,89 +530,21 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="D4" t="n">
-        <v>36521628895</v>
+        <v>39482011881</v>
       </c>
       <c r="E4" t="n">
         <v>402</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>'02</t>
-        </is>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Alice</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Corrente</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" t="n">
-        <v>14785236978</v>
-      </c>
-      <c r="E5" t="n">
-        <v>403</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>'03</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Israel</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Poupança</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>14785236900</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>404</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>'04</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>